<commit_message>
fix: corrige erro de indentação e medidas de validação
</commit_message>
<xml_diff>
--- a/output/resultados.xlsx
+++ b/output/resultados.xlsx
@@ -466,14 +466,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>90%</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>90%</t>
@@ -481,7 +481,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>80%</t>
         </is>
       </c>
     </row>
@@ -520,22 +520,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>56%</t>
+          <t>52%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>59%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>53%</t>
+          <t>49%</t>
         </is>
       </c>
     </row>
@@ -620,17 +620,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>224</t>
+          <t>225</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>93</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>89</t>
         </is>
       </c>
     </row>
@@ -642,22 +642,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>281</t>
+          <t>279</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>324</t>
+          <t>328</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>259</t>
+          <t>217</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>209</t>
         </is>
       </c>
     </row>
@@ -710,22 +710,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1222ms</t>
+          <t>1426ms</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1483ms</t>
+          <t>1572ms</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1835ms</t>
+          <t>1545ms</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>15038ms</t>
+          <t>1335ms</t>
         </is>
       </c>
     </row>
@@ -737,22 +737,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2225ms</t>
+          <t>2610ms</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2876ms</t>
+          <t>2473ms</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2090ms</t>
+          <t>2053ms</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>3153ms</t>
+          <t>2035ms</t>
         </is>
       </c>
     </row>
@@ -764,22 +764,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2388ms</t>
+          <t>2353ms</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4026ms</t>
+          <t>3534ms</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2767ms</t>
+          <t>3307ms</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2528ms</t>
+          <t>2349ms</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
         <v>77</v>
       </c>
       <c r="I2" t="n">
-        <v>1603</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="3">
@@ -919,7 +919,7 @@
         <v>183</v>
       </c>
       <c r="I3" t="n">
-        <v>1010</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="4">
@@ -958,7 +958,7 @@
         <v>135</v>
       </c>
       <c r="I4" t="n">
-        <v>1023</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="5">
@@ -997,7 +997,7 @@
         <v>77</v>
       </c>
       <c r="I5" t="n">
-        <v>2047</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="6">
@@ -1036,7 +1036,7 @@
         <v>80</v>
       </c>
       <c r="I6" t="n">
-        <v>1301</v>
+        <v>1430</v>
       </c>
     </row>
     <row r="7">
@@ -1075,7 +1075,7 @@
         <v>186</v>
       </c>
       <c r="I7" t="n">
-        <v>1687</v>
+        <v>1752</v>
       </c>
     </row>
     <row r="8">
@@ -1114,7 +1114,7 @@
         <v>138</v>
       </c>
       <c r="I8" t="n">
-        <v>1524</v>
+        <v>1604</v>
       </c>
     </row>
     <row r="9">
@@ -1153,7 +1153,7 @@
         <v>80</v>
       </c>
       <c r="I9" t="n">
-        <v>2754</v>
+        <v>1863</v>
       </c>
     </row>
     <row r="10">
@@ -1192,7 +1192,7 @@
         <v>71</v>
       </c>
       <c r="I10" t="n">
-        <v>68965</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="11">
@@ -1231,7 +1231,7 @@
         <v>177</v>
       </c>
       <c r="I11" t="n">
-        <v>1487</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="12">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NÃO URGENTE</t>
+          <t>POUCO URGENTE</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1261,16 +1261,16 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H12" t="n">
         <v>129</v>
       </c>
       <c r="I12" t="n">
-        <v>1225</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="13">
@@ -1309,7 +1309,7 @@
         <v>71</v>
       </c>
       <c r="I13" t="n">
-        <v>1328</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="14">
@@ -1330,25 +1330,25 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
+          <t>POUCO URGENTE</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>NÃO URGENTE</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>NÃO URGENTE</t>
-        </is>
-      </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G14" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H14" t="n">
         <v>71</v>
       </c>
       <c r="I14" t="n">
-        <v>1639</v>
+        <v>1983</v>
       </c>
     </row>
     <row r="15">
@@ -1369,25 +1369,25 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
+          <t>POUCO URGENTE</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
           <t>NÃO URGENTE</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>NÃO URGENTE</t>
-        </is>
-      </c>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G15" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H15" t="n">
         <v>177</v>
       </c>
       <c r="I15" t="n">
-        <v>2048</v>
+        <v>2314</v>
       </c>
     </row>
     <row r="16">
@@ -1426,7 +1426,7 @@
         <v>129</v>
       </c>
       <c r="I16" t="n">
-        <v>1209</v>
+        <v>1740</v>
       </c>
     </row>
     <row r="17">
@@ -1465,7 +1465,7 @@
         <v>71</v>
       </c>
       <c r="I17" t="n">
-        <v>1243</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="18">
@@ -1504,7 +1504,7 @@
         <v>73</v>
       </c>
       <c r="I18" t="n">
-        <v>1681</v>
+        <v>967</v>
       </c>
     </row>
     <row r="19">
@@ -1543,7 +1543,7 @@
         <v>179</v>
       </c>
       <c r="I19" t="n">
-        <v>1183</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="20">
@@ -1582,7 +1582,7 @@
         <v>131</v>
       </c>
       <c r="I20" t="n">
-        <v>1127</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="21">
@@ -1621,7 +1621,7 @@
         <v>73</v>
       </c>
       <c r="I21" t="n">
-        <v>1804</v>
+        <v>1845</v>
       </c>
     </row>
     <row r="22">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>{"sintoma":"dor abdominal","duracao":"2 dias","intensidade":"intensa"}</t>
+          <t>{"sintoma":"Dor abdominal","duracao":"2 dias","intensidade":"intensa"}</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1660,7 +1660,7 @@
         <v>57</v>
       </c>
       <c r="I22" t="n">
-        <v>3635</v>
+        <v>1955</v>
       </c>
     </row>
     <row r="23">
@@ -1699,7 +1699,7 @@
         <v>193</v>
       </c>
       <c r="I23" t="n">
-        <v>4290</v>
+        <v>3161</v>
       </c>
     </row>
     <row r="24">
@@ -1719,6 +1719,49 @@
         </is>
       </c>
       <c r="D24" t="inlineStr">
+        <is>
+          <t>{
+  "sintoma": "Dor abdominal",
+  "duracao": "2 dias",
+  "intensidade": "intensa"
+}</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>{'sintoma': 'dor abdominal', 'duracao': '2 dias', 'intensidade': 'intensa'}</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="n">
+        <v>140</v>
+      </c>
+      <c r="H24" t="n">
+        <v>108</v>
+      </c>
+      <c r="I24" t="n">
+        <v>3304</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>extracao_dados_paciente</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>role_prompting</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Dor abdominal intensa há 2 dias</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
         <is>
           <t>{
   "sintoma": "dor abdominal",
@@ -1727,49 +1770,6 @@
 }</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>{'sintoma': 'dor abdominal', 'duracao': '2 dias', 'intensidade': 'intensa'}</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" t="n">
-        <v>140</v>
-      </c>
-      <c r="H24" t="n">
-        <v>108</v>
-      </c>
-      <c r="I24" t="n">
-        <v>1937</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>extracao_dados_paciente</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>role_prompting</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Dor abdominal intensa há 2 dias</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>{
-  "sintoma": "dor abdominal",
-  "duracao": "2 dias",
-  "intensidade": "intensa"
-}</t>
-        </is>
-      </c>
       <c r="E25" t="inlineStr">
         <is>
           <t>{'sintoma': 'dor abdominal', 'duracao': '2 dias', 'intensidade': 'intensa'}</t>
@@ -1785,7 +1785,7 @@
         <v>57</v>
       </c>
       <c r="I25" t="n">
-        <v>2020</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="26">
@@ -1805,6 +1805,123 @@
         </is>
       </c>
       <c r="D26" t="inlineStr">
+        <is>
+          <t>{"sintoma":"tontura","duracao":"desde esta manhã","intensidade":"leve"}</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>{'sintoma': 'tontura', 'duracao': 'algumas horas', 'intensidade': 'leve'}</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G26" t="n">
+        <v>84</v>
+      </c>
+      <c r="H26" t="n">
+        <v>58</v>
+      </c>
+      <c r="I26" t="n">
+        <v>2367</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>extracao_dados_paciente</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>few_shot</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Tontura leve desde esta manhã</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>{"sintoma": "tontura", "duracao": "1 dia", "intensidade": "leve"}</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>{'sintoma': 'tontura', 'duracao': 'algumas horas', 'intensidade': 'leve'}</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G27" t="n">
+        <v>221</v>
+      </c>
+      <c r="H27" t="n">
+        <v>194</v>
+      </c>
+      <c r="I27" t="n">
+        <v>2896</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>extracao_dados_paciente</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>chain_of_thought</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Tontura leve desde esta manhã</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>{"sintoma":"tontura","duracao":"desde esta manhã","intensidade":"leve"}</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>{'sintoma': 'tontura', 'duracao': 'algumas horas', 'intensidade': 'leve'}</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G28" t="n">
+        <v>135</v>
+      </c>
+      <c r="H28" t="n">
+        <v>109</v>
+      </c>
+      <c r="I28" t="n">
+        <v>2107</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>extracao_dados_paciente</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>role_prompting</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Tontura leve desde esta manhã</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
         <is>
           <t>{
   "sintoma": "tontura",
@@ -1813,127 +1930,6 @@
 }</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>{'sintoma': 'tontura', 'duracao': 'algumas horas', 'intensidade': 'leve'}</t>
-        </is>
-      </c>
-      <c r="F26" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="G26" t="n">
-        <v>94</v>
-      </c>
-      <c r="H26" t="n">
-        <v>58</v>
-      </c>
-      <c r="I26" t="n">
-        <v>2296</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>extracao_dados_paciente</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>few_shot</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Tontura leve desde esta manhã</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>{"sintoma": "tontura", "duracao": "hoje", "intensidade": "leve"}</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>{'sintoma': 'tontura', 'duracao': 'algumas horas', 'intensidade': 'leve'}</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="G27" t="n">
-        <v>221</v>
-      </c>
-      <c r="H27" t="n">
-        <v>194</v>
-      </c>
-      <c r="I27" t="n">
-        <v>2632</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>extracao_dados_paciente</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>chain_of_thought</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Tontura leve desde esta manhã</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>{"sintoma":"tontura","duracao":"desde esta manhã","intensidade":"leve"}</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>{'sintoma': 'tontura', 'duracao': 'algumas horas', 'intensidade': 'leve'}</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="G28" t="n">
-        <v>135</v>
-      </c>
-      <c r="H28" t="n">
-        <v>109</v>
-      </c>
-      <c r="I28" t="n">
-        <v>1750</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>extracao_dados_paciente</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>role_prompting</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Tontura leve desde esta manhã</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>{
-  "sintoma": "tontura",
-  "duracao": "desde esta manhã",
-  "intensidade": "leve"
-}</t>
-        </is>
-      </c>
       <c r="E29" t="inlineStr">
         <is>
           <t>{'sintoma': 'tontura', 'duracao': 'algumas horas', 'intensidade': 'leve'}</t>
@@ -1949,7 +1945,7 @@
         <v>58</v>
       </c>
       <c r="I29" t="n">
-        <v>2355</v>
+        <v>1597</v>
       </c>
     </row>
     <row r="30">
@@ -1992,7 +1988,7 @@
         <v>59</v>
       </c>
       <c r="I30" t="n">
-        <v>2352</v>
+        <v>1854</v>
       </c>
     </row>
     <row r="31">
@@ -2031,7 +2027,7 @@
         <v>195</v>
       </c>
       <c r="I31" t="n">
-        <v>2269</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="32">
@@ -2051,6 +2047,45 @@
         </is>
       </c>
       <c r="D32" t="inlineStr">
+        <is>
+          <t>{"sintoma":"Falta de ar","duracao":"3 horas","intensidade":"moderada"}</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>{'sintoma': 'falta de ar', 'duracao': '3 horas', 'intensidade': 'moderada'}</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="n">
+        <v>134</v>
+      </c>
+      <c r="H32" t="n">
+        <v>110</v>
+      </c>
+      <c r="I32" t="n">
+        <v>1737</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>extracao_dados_paciente</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>role_prompting</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Falta de ar moderada há 3 horas</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
         <is>
           <t>{
   "sintoma": "Falta de ar",
@@ -2059,49 +2094,6 @@
 }</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>{'sintoma': 'falta de ar', 'duracao': '3 horas', 'intensidade': 'moderada'}</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G32" t="n">
-        <v>144</v>
-      </c>
-      <c r="H32" t="n">
-        <v>110</v>
-      </c>
-      <c r="I32" t="n">
-        <v>2396</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>extracao_dados_paciente</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>role_prompting</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Falta de ar moderada há 3 horas</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>{
-  "sintoma": "Falta de ar",
-  "duracao": "3 horas",
-  "intensidade": "moderada"
-}</t>
-        </is>
-      </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>{'sintoma': 'falta de ar', 'duracao': '3 horas', 'intensidade': 'moderada'}</t>
@@ -2117,7 +2109,7 @@
         <v>59</v>
       </c>
       <c r="I33" t="n">
-        <v>1681</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="34">
@@ -2137,88 +2129,6 @@
         </is>
       </c>
       <c r="D34" t="inlineStr">
-        <is>
-          <t>{
-  "sintoma": "dor de garganta com dificuldade para engolir",
-  "duracao": "4 dias",
-  "intensidade": "forte"
-}</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>{'sintoma': 'dor de garganta', 'duracao': '4 dias', 'intensidade': 'forte'}</t>
-        </is>
-      </c>
-      <c r="F34" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" t="n">
-        <v>108</v>
-      </c>
-      <c r="H34" t="n">
-        <v>66</v>
-      </c>
-      <c r="I34" t="n">
-        <v>4095</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>extracao_dados_paciente</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>few_shot</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Dor de garganta forte há 4 dias com dificuldade para engolir</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>{"sintoma": "dor de garganta", "duracao": "4 dias", "intensidade": "forte"}</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>{'sintoma': 'dor de garganta', 'duracao': '4 dias', 'intensidade': 'forte'}</t>
-        </is>
-      </c>
-      <c r="F35" t="n">
-        <v>1</v>
-      </c>
-      <c r="G35" t="n">
-        <v>231</v>
-      </c>
-      <c r="H35" t="n">
-        <v>202</v>
-      </c>
-      <c r="I35" t="n">
-        <v>2457</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>extracao_dados_paciente</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>chain_of_thought</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Dor de garganta forte há 4 dias com dificuldade para engolir</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
         <is>
           <t>{
   "sintoma": "dor de garganta",
@@ -2227,6 +2137,88 @@
 }</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>{'sintoma': 'dor de garganta', 'duracao': '4 dias', 'intensidade': 'forte'}</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="n">
+        <v>100</v>
+      </c>
+      <c r="H34" t="n">
+        <v>66</v>
+      </c>
+      <c r="I34" t="n">
+        <v>1951</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>extracao_dados_paciente</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>few_shot</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Dor de garganta forte há 4 dias com dificuldade para engolir</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>{"sintoma": "dor de garganta", "duracao": "4 dias", "intensidade": "forte"}</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>{'sintoma': 'dor de garganta', 'duracao': '4 dias', 'intensidade': 'forte'}</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="n">
+        <v>231</v>
+      </c>
+      <c r="H35" t="n">
+        <v>202</v>
+      </c>
+      <c r="I35" t="n">
+        <v>2483</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>extracao_dados_paciente</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>chain_of_thought</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Dor de garganta forte há 4 dias com dificuldade para engolir</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>{
+  "sintoma": "Dor de garganta",
+  "duracao": "4 dias",
+  "intensidade": "forte"
+}</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
           <t>{'sintoma': 'dor de garganta', 'duracao': '4 dias', 'intensidade': 'forte'}</t>
@@ -2242,7 +2234,7 @@
         <v>117</v>
       </c>
       <c r="I36" t="n">
-        <v>1943</v>
+        <v>3453</v>
       </c>
     </row>
     <row r="37">
@@ -2285,7 +2277,7 @@
         <v>66</v>
       </c>
       <c r="I37" t="n">
-        <v>1637</v>
+        <v>2046</v>
       </c>
     </row>
     <row r="38">
@@ -2328,7 +2320,7 @@
         <v>60</v>
       </c>
       <c r="I38" t="n">
-        <v>3388</v>
+        <v>2046</v>
       </c>
     </row>
     <row r="39">
@@ -2349,7 +2341,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>{"sintoma": "náusea", "duracao": "1 dia", "intensidade": "fraca"}</t>
+          <t>{"sintoma": "náusea", "duracao": "após o almoço", "intensidade": "fraca"}</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2361,13 +2353,13 @@
         <v>0.67</v>
       </c>
       <c r="G39" t="n">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="H39" t="n">
         <v>196</v>
       </c>
       <c r="I39" t="n">
-        <v>2731</v>
+        <v>2159</v>
       </c>
     </row>
     <row r="40">
@@ -2388,7 +2380,11 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>{"sintoma":"náusea","duracao":"","intensidade":"fraca"}</t>
+          <t>{
+  "sintoma": "náusea",
+  "duracao": null,
+  "intensidade": "fraca"
+}</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2400,13 +2396,13 @@
         <v>0.67</v>
       </c>
       <c r="G40" t="n">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="H40" t="n">
         <v>111</v>
       </c>
       <c r="I40" t="n">
-        <v>3099</v>
+        <v>2447</v>
       </c>
     </row>
     <row r="41">
@@ -2428,8 +2424,8 @@
       <c r="D41" t="inlineStr">
         <is>
           <t>{
-  "sintoma": "Náusea",
-  "duracao": "após o almoço",
+  "sintoma": "náusea",
+  "duracao": null,
   "intensidade": "fraca"
 }</t>
         </is>
@@ -2443,13 +2439,13 @@
         <v>0.67</v>
       </c>
       <c r="G41" t="n">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="H41" t="n">
         <v>60</v>
       </c>
       <c r="I41" t="n">
-        <v>2759</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="42">
@@ -2470,11 +2466,11 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>- Paciente: Maria, 62 anos, diabética tipo 2  
-- Queixa principal: tontura e visão turva há 1 hora  
-- Glicemia capilar: 320 mg/dL (hiperglicemia)  
-- Pressão arterial: 140/90 mmHg  
-- Necessário monitoramento glicêmico, avaliação neurológica e ajuste de terapia antidiabética.</t>
+          <t>- Paciente: Maria, 62 anos, diabética conhecida.  
+- Queixa principal: tontura e visão turva há 1 hora.  
+- Glicemia capilar: 320 mg/dL (hiperglicemia).  
+- Pressão arterial: 140/90 mmHg.  
+- Necessário: avaliação rápida, correção glicêmica (insulina IV/SC), monitoramento neurológico e hemodinâmico, investigar causa da hiperglicemia (infecção, medicação).</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2486,13 +2482,13 @@
         <v>0.75</v>
       </c>
       <c r="G42" t="n">
-        <v>190</v>
+        <v>216</v>
       </c>
       <c r="H42" t="n">
         <v>86</v>
       </c>
       <c r="I42" t="n">
-        <v>2352</v>
+        <v>1939</v>
       </c>
     </row>
     <row r="43">
@@ -2515,9 +2511,9 @@
         <is>
           <t>• Mulher, 62 anos, diabética  
 • Tontura e visão turva há 1 h  
-• Glicemia: 320 mg/dL  
-• PA: 140/90 mmHg  
-• Avaliar hiperglicemia aguda (cetoacidose), iniciar fluidos + insulina, monitorar cetonas e sinais vitais</t>
+• Glicemia capilar: 320 mg/dL  
+• Pressão arterial: 140/90 mmHg  
+• Suspeita de hiperglicemia descompensada – iniciar controle glicêmico e monitorar sinais neurológicos</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2535,7 +2531,7 @@
         <v>243</v>
       </c>
       <c r="I43" t="n">
-        <v>5015</v>
+        <v>2651</v>
       </c>
     </row>
     <row r="44">
@@ -2556,11 +2552,11 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>- Paciente: Maria, 62 anos, sexo feminino, diabética tipo 2.  
-- Queixa: tontura e visão turva, início há 1 hora.  
+          <t>- Paciente: Maria, 62 anos, sexo feminino, história de diabetes mellitus.  
+- Queixa principal: tontura e visão turva iniciadas há 1 hora.  
 - Glicemia capilar: 320 mg/dL (hiperglicemia).  
 - Pressão arterial: 140/90 mmHg.  
-- Prioridade: correção rápida da hiperglicemia e avaliação de causa neurológica/vascular.</t>
+- Prioridade: controle glicêmico urgente + avaliação neurológica/vascular antes de alta.</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2569,16 +2565,16 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="G44" t="n">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="H44" t="n">
         <v>148</v>
       </c>
       <c r="I44" t="n">
-        <v>1729</v>
+        <v>1869</v>
       </c>
     </row>
     <row r="45">
@@ -2599,11 +2595,11 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>- **Paciente:** Maria, 62 anos, diabética tipo 2.  
+          <t>- **Paciente:** Maria, 62 anos, história de diabetes mellitus.  
 - **Queixa principal:** Tontura e visão turva há 1 hora.  
 - **Sinais vitais:** PA 140/90 mmHg; glicemia capilar 320 mg/dL.  
-- **Risco imediato:** Hiperglicemia com possível descompensação osmótica/cefálica; necessidade de avaliação neurológica e correção de glicemia.  
-- **Ações urgentes:** Monitorização contínua, reposição de fluidos, iniciar correção de glicemia (insulina IV conforme protocolo), solicitar exames laboratoriais (eletrólitos, cetonas, hemograma) e avaliação neurológica.</t>
+- **Risco imediato:** Hiperglicemia significativa em diabético → risco de descompensação hiperosmolar; sintoma neurológico (tontura/visão).  
+- **Triagem Manchester:** Categoria **Orange** (urgência muito alta – atendimento dentro de 10 min).</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2612,16 +2608,16 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="G45" t="n">
-        <v>272</v>
+        <v>233</v>
       </c>
       <c r="H45" t="n">
         <v>86</v>
       </c>
       <c r="I45" t="n">
-        <v>2468</v>
+        <v>3460</v>
       </c>
     </row>
     <row r="46">
@@ -2643,10 +2639,10 @@
       <c r="D46" t="inlineStr">
         <is>
           <t>- Paciente: Pedro, 8 anos, histórico de asma.  
-- Queixa: chiado no peito e dificuldade respiratória há 30 min.  
-- Sinais vitais: SpO₂ = 91 % (hipoxemia).  
-- Avaliação: provável exacerbação asmática aguda.  
-- Necessário: oxigênio suplementar, broncodilatador de curta ação e avaliação para possível terapia sistêmica.</t>
+- Queixa principal: chiado no peito e dificuldade respiratória há 30 min.  
+- Saturação de oxigênio: SpO₂ = 91 % (hipoxemia leve).  
+- Sinais vitais: frequência respiratória aumentada, esforço inspiratório perceptível.  
+- Necessário: avaliação rápida, suporte de oxigênio, broncodilatador de ação rápida e monitoramento contínuo.</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2655,16 +2651,16 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="G46" t="n">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="H46" t="n">
         <v>80</v>
       </c>
       <c r="I46" t="n">
-        <v>1839</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="47">
@@ -2686,10 +2682,10 @@
       <c r="D47" t="inlineStr">
         <is>
           <t>• Menino, 8 anos, histórico de asma  
-• Chiado e dispneia há 30 min  
-• Saturação de O₂ ↓ 91 % (hipoxemia)  
-• Iniciar oxigênio suplementar + nebulização com broncodilatador  
-• Monitorar resposta, frequência respiratória e sinais de fadiga</t>
+• Chiado no peito e dispneia há 30 min  
+• Saturação de O₂ 91 % (hipoxemia)  
+• Avaliar necessidade de oxigênio e broncodilatador de curta ação  
+• Monitorar resposta ao tratamento e sinais de fadiga respiratória</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2701,13 +2697,13 @@
         <v>0.2</v>
       </c>
       <c r="G47" t="n">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="H47" t="n">
         <v>237</v>
       </c>
       <c r="I47" t="n">
-        <v>3481</v>
+        <v>6604</v>
       </c>
     </row>
     <row r="48">
@@ -2729,10 +2725,10 @@
       <c r="D48" t="inlineStr">
         <is>
           <t>- Paciente: Pedro, 8 anos, sexo masculino, histórico de asma.  
-- Queixa: chiado no peito e dificuldade respiratória iniciados há 30 min.  
+- Queixa: chiado no peito e dificuldade respiratória há 30 min.  
 - Saturação de oxigênio: SpO₂ = 91 % (hipoxemia).  
-- Sinais vitais: taquipneia (não informada), uso de musculatura acessória provável.  
-- Prioridade: iniciar broncodilatador de curta ação + oxigênio suplementar; monitorar resposta e considerar escalonamento de terapia.</t>
+- Sinais vitais: (não informados) → monitorar frequência respiratória, frequência cardíaca e pressão arterial.  
+- Prioridade: iniciar suporte de oxigênio, avaliar necessidade de broncodilatador de curta ação e considerar escalonamento de terapia para crise asmática.</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2741,16 +2737,16 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="G48" t="n">
-        <v>284</v>
+        <v>293</v>
       </c>
       <c r="H48" t="n">
         <v>142</v>
       </c>
       <c r="I48" t="n">
-        <v>1944</v>
+        <v>2047</v>
       </c>
     </row>
     <row r="49">
@@ -2772,10 +2768,10 @@
       <c r="D49" t="inlineStr">
         <is>
           <t>- Paciente: Pedro, 8 anos, histórico de asma.  
-- Queixa principal: chiado no peito + dispneia há 30 min.  
-- Sinais vitais: SpO₂ = 91 % (oxigenação comprometida), frequência respiratória aumentada (não informada).  
-- Avaliação rápida (Manchester): categoria **Urgente (Amarelo)** – risco de deterioração respiratória.  
-- Plano imediato: oxigênio suplementar (≥ 2 L/min), nebulização com broncodilatador + corticoide, monitorização contínua e preparo para suporte ventilatório se necessário.</t>
+- Queixa principal: chiado no peito + dificuldade respiratória há ≈ 30 min.  
+- Sinais vitais: SpO₂ = 91 % (oxigenação baixa), frequência respiratória aumentada (não informada).  
+- Classificação Manchester: **Urgente (Amarelo)** – risco de deterioração respiratória.  
+- Recomendações imediatas: iniciar oxigênio suplementar (≥ 2 L/min), nebulização com broncodilatador de curta ação + corticoide, monitorar SpO₂ e sinais vitais, preparar suporte avançado de via aérea se piorar.</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2787,13 +2783,13 @@
         <v>0.2</v>
       </c>
       <c r="G49" t="n">
-        <v>246</v>
+        <v>271</v>
       </c>
       <c r="H49" t="n">
         <v>80</v>
       </c>
       <c r="I49" t="n">
-        <v>2149</v>
+        <v>2765</v>
       </c>
     </row>
     <row r="50">
@@ -2814,158 +2810,158 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
+          <t>- Paciente: Ana, 28 anos, gestante de 32 semanas.  
+- Queixa principal: dor abdominal intensa + sangramento vaginal.  
+- Sinais vitais (a confirmar): pressão arterial, frequência cardíaca, saturação.  
+- Principais hipóteses diagnósticas: descolamento prematuro de placenta, trabalho de parto prematuro, ruptura uterina.  
+- Condutas urgentes: monitorização fetal, hemograma, tipagem sanguínea, iniciar suporte hemodinâmico e preparar equipe obstétrica para possível intervenção.</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Emergência obstétrica</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G50" t="n">
+        <v>209</v>
+      </c>
+      <c r="H50" t="n">
+        <v>67</v>
+      </c>
+      <c r="I50" t="n">
+        <v>3586</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>sumarizacao_prontuario</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>few_shot</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Paciente Ana, 28 anos, grávida 32 semanas, dor abdominal intensa e sangramento vaginal</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>• Mulher, 28 anos, gestante 32 semanas  
+• Dor abdominal intensa  
+• Sangramento vaginal (presença de fluxo)  
+• Suspeita de emergência obstétrica (ex.: descolamento de placenta ou placenta prévia)  
+• Avaliar sinais vitais, exame pélvico, ultrassom obstétrico e preparar para manejo de hemorragia/parto emergencial</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Emergência obstétrica</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" t="n">
+        <v>326</v>
+      </c>
+      <c r="H51" t="n">
+        <v>224</v>
+      </c>
+      <c r="I51" t="n">
+        <v>2496</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>sumarizacao_prontuario</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>chain_of_thought</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Paciente Ana, 28 anos, grávida 32 semanas, dor abdominal intensa e sangramento vaginal</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>- Paciente: Ana, 28 anos, gestante de 32 semanas.  
+- Queixa principal: dor abdominal intensa + sangramento vaginal.  
+- Evolução: início súbito (tempo não especificado), dor contínua.  
+- Sinais de alerta: risco de descolamento prematuro de placenta ou trabalho de parto precoce.  
+- Necessário: avaliação obstétrica urgente, monitorização fetal, hemograma, tipagem sanguínea e preparo para possível intervenção.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Emergência obstétrica</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G52" t="n">
+        <v>257</v>
+      </c>
+      <c r="H52" t="n">
+        <v>129</v>
+      </c>
+      <c r="I52" t="n">
+        <v>1900</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>sumarizacao_prontuario</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>role_prompting</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Paciente Ana, 28 anos, grávida 32 semanas, dor abdominal intensa e sangramento vaginal</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
           <t>- Paciente: Ana, 28 anos, gestante de 32 semanas de gestação.  
 - Queixa principal: dor abdominal intensa + sangramento vaginal.  
-- Sinais vitais (a confirmar): pressão arterial, frequência cardíaca, saturação e avaliação fetal.  
-- Suspeita de complicação obstétrica: ruptura prematura de membranas, placenta prévia ou descolamento placentário.  
-- Medidas imediatas: monitorização materno‑fetal, acesso venoso, preparo para avaliação ultrassonográfica e possível intervenção obstétrica de urgência.</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
+- Sinais vitais (se disponíveis): monitorar pressão arterial, frequência cardíaca, saturação e temperatura.  
+- Suspeita de complicação obstétrica (ex.: descolamento prematuro de placenta ou trabalho de parto prematuro) – risco de hemorragia e comprometimento fetal.  
+- Prioridade Manchester: **Red (imediata)** – necessidade de avaliação obstétrica urgente e suporte hemodinâmico.</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>Emergência obstétrica</t>
         </is>
       </c>
-      <c r="F50" t="n">
+      <c r="F53" t="n">
         <v>0.5</v>
       </c>
-      <c r="G50" t="n">
-        <v>213</v>
-      </c>
-      <c r="H50" t="n">
-        <v>67</v>
-      </c>
-      <c r="I50" t="n">
-        <v>2868</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>sumarizacao_prontuario</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>few_shot</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Paciente Ana, 28 anos, grávida 32 semanas, dor abdominal intensa e sangramento vaginal</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>• Mulher, 28 anos, gestante 32 semanas  
-• Dor abdominal intensa  
-• Sangramento vaginal  
-• Avaliar sinais de gravidade (PA, FC, volume de sangramento, contrações)  
-• Monitorar fetal (cardiotocografia) e preparar manejo obstétrico urgente</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Emergência obstétrica</t>
-        </is>
-      </c>
-      <c r="F51" t="n">
-        <v>0</v>
-      </c>
-      <c r="G51" t="n">
-        <v>298</v>
-      </c>
-      <c r="H51" t="n">
-        <v>224</v>
-      </c>
-      <c r="I51" t="n">
-        <v>3491</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>sumarizacao_prontuario</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>chain_of_thought</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Paciente Ana, 28 anos, grávida 32 semanas, dor abdominal intensa e sangramento vaginal</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>- **Paciente:** Ana, 28 anos, gestante, 32 semanas de gestação.  
-- **Queixa principal:** Dor abdominal intensa de início súbito.  
-- **Sintoma associado:** Sangramento vaginal (quantidade não especificada).  
-- **Urgência:** Suspeita de descolamento prematuro de placenta ou trabalho de parto prematuro – requer avaliação obstétrica imediata e monitorização fetal.  
-- **Ações imediatas:** Monitorar sinais vitais, iniciar acesso venoso, coletar hemograma, tipagem e cruzamento sanguíneo, avaliar via ultrassonografia obstétrica e preparar para possível transferência para unidade de alto risco.</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Emergência obstétrica</t>
-        </is>
-      </c>
-      <c r="F52" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G52" t="n">
-        <v>303</v>
-      </c>
-      <c r="H52" t="n">
-        <v>129</v>
-      </c>
-      <c r="I52" t="n">
-        <v>2546</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>sumarizacao_prontuario</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>role_prompting</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Paciente Ana, 28 anos, grávida 32 semanas, dor abdominal intensa e sangramento vaginal</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>- Paciente: Ana, 28 anos, gestante 32 semanas de gestação.  
-- Queixa principal: dor abdominal intensa + sangramento vaginal (quantidade não especificada).  
-- Sinais vitais (a confirmar): pressão arterial, frequência cardíaca, saturação e frequência uterina.  
-- Suspeita de complicação obstétrica (abruptio placentae ou trabalho de parto prematuro) – iniciar monitorização fetal e uterina.  
-- Ações imediatas: garantir via aérea e hemodinâmica, iniciar acesso venoso, solicitar hemograma, tipagem sanguínea + cross‑match, ultrassonografia obstétrica e preparar equipe de obstetrícia para possível parto de emergência.</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Emergência obstétrica</t>
-        </is>
-      </c>
-      <c r="F53" t="n">
-        <v>1</v>
-      </c>
       <c r="G53" t="n">
-        <v>250</v>
+        <v>218</v>
       </c>
       <c r="H53" t="n">
         <v>67</v>
       </c>
       <c r="I53" t="n">
-        <v>3173</v>
+        <v>2660</v>
       </c>
     </row>
     <row r="54">
@@ -2987,10 +2983,10 @@
       <c r="D54" t="inlineStr">
         <is>
           <t>- Paciente: Carlos, 55 anos  
-- Queixa: fala arrastada e fraqueza no lado direito do corpo  
+- Queixa principal: fala arrastada e fraqueza no lado direito  
 - Início dos sintomas: há aproximadamente 2 horas  
-- Suspeita clínica: AVC isquêmico (possível hemiparesia esquerda)  
-- Prioridade: avaliação neurológica, NIHSS, TC de crânio sem contraste e considerar trombólise se elegível.</t>
+- Sinais neurológicos: hemiparesia direita, disartria; sem relato de dor de cabeça ou perda de consciência  
+- Suspeita clínica: AVC isquêmico agudo – necessidade de avaliação neuroimagiológica urgente e início de terapia trombolítica se elegível.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -3002,13 +2998,13 @@
         <v>1</v>
       </c>
       <c r="G54" t="n">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="H54" t="n">
         <v>74</v>
       </c>
       <c r="I54" t="n">
-        <v>3175</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="55">
@@ -3031,9 +3027,9 @@
         <is>
           <t>• Homem, 55 anos, início súbito há 2 h  
 • Fala arrastada e fraqueza do lado direito do corpo  
-• Suspeita de AVC isquêmico (possível hemisfério esquerdo)  
-• Avaliar escala de AVC (NIHSS), pressão arterial e glicemia  
-• Iniciar protocolo de AVC: TC de crânio urgente, considerar trombólise se elegível</t>
+• Suspeita de AVC isquêmico agudo  
+• Avaliar NIHSS, pressão arterial e glicemia imediatamente  
+• Considerar TC de crânio e iniciar trombólise se elegível</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3045,13 +3041,13 @@
         <v>1</v>
       </c>
       <c r="G55" t="n">
-        <v>338</v>
+        <v>319</v>
       </c>
       <c r="H55" t="n">
         <v>231</v>
       </c>
       <c r="I55" t="n">
-        <v>3584</v>
+        <v>2359</v>
       </c>
     </row>
     <row r="56">
@@ -3072,11 +3068,11 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>- 55 anos, masculino (Carlos)  
-- Chegou ao pronto‑socorro há 2 h com fala arrastada e fraqueza no lado direito do corpo  
-- Sinais neurológicos: hemiparesia direita (braço e perna), possível déficit sensorial; provável escala de Glasgow 14‑15  
-- Suspeita de AVC isquêmico agudo – tempo de início &lt; 4,5 h, candidato à trombólise se exames permitirem  
-- Ações imediatas: monitorização de sinais vitais, glicemia capilar, TC de crânio sem contraste, painel de coagulação e iniciar protocolo de AVC.</t>
+          <t>- **Paciente:** Carlos, 55 anos, masculino  
+- **Queixa principal:** fala arrastada + fraqueza do lado direito do corpo  
+- **Tempo de evolução:** início há aproximadamente 2 horas  
+- **Sinais de alerta:** suspeita de AVC (sintomas focais neurológicos agudos)  
+- **Urgência:** necessidade de avaliação neurológica imediata, escala de AVC, TC de crânio e início de terapia trombolítica se indicado.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3088,13 +3084,13 @@
         <v>1</v>
       </c>
       <c r="G56" t="n">
-        <v>305</v>
+        <v>265</v>
       </c>
       <c r="H56" t="n">
         <v>136</v>
       </c>
       <c r="I56" t="n">
-        <v>3880</v>
+        <v>1962</v>
       </c>
     </row>
     <row r="57">
@@ -3115,11 +3111,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>- **Paciente:** Carlos, 55 anos, masculino  
-- **Queixa principal:** Fala arrastada + fraqueza no lado direito do corpo  
-- **Tempo de evolução:** 2 horas desde o início dos sintomas  
-- **Sinais de alerta:** Possível AVC agudo (déficit neurológico focal) – prioridade Manchester **Red** (imediata)  
-- **Ações iniciais:** Avaliar via ABC, monitorização contínua, oxigênio se SpO₂ &lt; 94 %, acesso venoso, iniciar escala de AVC (NIHSS) e preparar para imagem cerebral urgente (TC/angiografia).</t>
+          <t>- Paciente: Carlos, 55 anos, masculino</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3128,16 +3120,16 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>0.67</v>
+        <v>0</v>
       </c>
       <c r="G57" t="n">
-        <v>237</v>
+        <v>88</v>
       </c>
       <c r="H57" t="n">
         <v>74</v>
       </c>
       <c r="I57" t="n">
-        <v>2970</v>
+        <v>4174</v>
       </c>
     </row>
     <row r="58">
@@ -3158,11 +3150,11 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>- Paciente: Lúcia, 40 anos.  
-- Alergia conhecida: dipirona (metamizol).  
-- Exposição: ingestão acidental de dipirona.  
-- Manifestação clínica: urticária generalizada (lesões eritematosas pruriginosas).  
-- Conduta recomendada: suspensão do agente, antihistamínico de primeira linha, monitorar sinais de anafilaxia e considerar adrenalina se houver progressão.</t>
+          <t>- **Paciente:** Lúcia, 40 anos  
+- **Alergia conhecida:** Dipirona (metamizol)  
+- **Evento:** Ingestão acidental de dipirona hoje  
+- **Manifestação atual:** Urticária generalizada, sem comprometimento respiratório aparente  
+- **Conduta recomendada:** Monitorar sinais vitais, administrar antihistamínico (ex.: cetirizina) e, se houver piora ou sinais de anafilaxia, iniciar adrenalina IM e suporte avançado.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3174,13 +3166,13 @@
         <v>0</v>
       </c>
       <c r="G58" t="n">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="H58" t="n">
         <v>77</v>
       </c>
       <c r="I58" t="n">
-        <v>2406</v>
+        <v>2177</v>
       </c>
     </row>
     <row r="59">
@@ -3203,9 +3195,9 @@
         <is>
           <t>• Mulher, 40 anos, alergia conhecida à dipirona  
 • Ingestão acidental de dipirona  
-• Urticária generalizada, sem sinais de comprometimento respiratório imediato  
-• Monitorar PA, frequência respiratória e sinais de anafilaxia  
-• Iniciar antihistamínico e ter adrenalina à mão caso haja piora</t>
+• Urticária generalizada, sem comprometimento respiratório aparente  
+• Administrar anti‑histamínico (ex.: difenidramina) e observar evolução  
+• Monitorar sinais de anafilaxia; ter epinefrina à mão caso haja piora</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3217,13 +3209,13 @@
         <v>0</v>
       </c>
       <c r="G59" t="n">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="H59" t="n">
         <v>234</v>
       </c>
       <c r="I59" t="n">
-        <v>4560</v>
+        <v>3559</v>
       </c>
     </row>
     <row r="60">
@@ -3244,11 +3236,11 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>- Paciente: Lúcia, 40 anos, sexo feminino.  
-- Alergia conhecida: dipirona (reação prévia).  
-- Exposição: ingestão acidental de dipirona há &lt;1 h.  
-- Sinais atuais: urticária generalizada, sem comprometimento respiratório aparente.  
-- Medidas urgentes: monitorar via aérea, administrar antihistamínico/epinefrina conforme protocolo de anafilaxia.</t>
+          <t>- **Paciente:** Lúcia, 40 anos, sexo feminino.  
+- **Histórico de alergia:** Hipersensibilidade conhecida à dipirona.  
+- **Evento atual:** Ingestão acidental de dipirona; início de urticária generalizada.  
+- **Sinais clínicos:** Lesões urticariformes disseminadas, sem relato de edema de lábios ou comprometimento respiratório até o momento.  
+- **Conduta urgente:** Monitorar vias aéreas; iniciar antihistamínico (cetirizina ou difenidramina) e, se houver piora ou sinais de anafilaxia, administrar epinefrina 0,3 mg IM; observar por pelo menos 2 h.</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3257,16 +3249,16 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>0.33</v>
+        <v>0</v>
       </c>
       <c r="G60" t="n">
-        <v>255</v>
+        <v>324</v>
       </c>
       <c r="H60" t="n">
         <v>139</v>
       </c>
       <c r="I60" t="n">
-        <v>1841</v>
+        <v>3987</v>
       </c>
     </row>
     <row r="61">
@@ -3289,9 +3281,9 @@
         <is>
           <t>- Paciente: Lúcia, 40 anos; alergia conhecida à dipirona.  
 - Exposição: ingestão acidental de dipirona há ~30 min.  
-- Sinais clínicos: urticária maculopapular generalizada, prurido intenso; sem edema de vias aéreas nem comprometimento respiratório aparente.  
-- Avaliação inicial: PA 120/80 mmHg, FC 92 bpm, SpO₂ 98% em ar ambiente, sem sibilos ou dificuldade respiratória.  
-- Conduta imediata: administração de antihistamínico de ação rápida (ex.: cetirizina 10 mg VO) + observação por ≥1 h; preparo de adrenalina 0,3 mg IM caso evolua para anafilaxia; notificar equipe de alergologia.</t>
+- Sinais atuais: urticária maculopapular generalizada, sem edema de vias aéreas nem prurido intenso.  
+- VSR: PA 120/80 mmHg, FC 92 bpm, SpO₂ 98% em ar ambiente, sem dispneia.  
+- Medidas iniciais: suspensão do agente, administração IM de adrenalina 0,3 mg (1 mL 1:1000) + antihistamínico (cetirizina 10 mg PO) e observação por 2 h; monitorar sinais de anafilaxia.</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3303,13 +3295,13 @@
         <v>0</v>
       </c>
       <c r="G61" t="n">
-        <v>292</v>
+        <v>277</v>
       </c>
       <c r="H61" t="n">
         <v>77</v>
       </c>
       <c r="I61" t="n">
-        <v>3073</v>
+        <v>3477</v>
       </c>
     </row>
   </sheetData>

</xml_diff>